<commit_message>
feat: full system - notifications, employee restrictions, dark mode removal, department scoping
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Notification Triggers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Selective Merge" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -835,4 +836,436 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>File / Component</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Action Taken</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Rationale / Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>frontend/src/styles/theme.css</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Category B (Light Mode Tokens)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Merged (:root Light Mode Tokens)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Updated Light Mode colors (--bg-main: #f7f8fa, --accent-color: #10b981). Dark Mode tokens preserved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>frontend/src/components/Button/Button.css</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Category B (Light Mode Styling)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Merged (Primary Button Style)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Updated Primary Button to Vibrant Emerald (#10b981 background, #0b0c10 text).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>frontend/src/components/Input/Input.css</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Category B (Light Mode Styling)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Merged (Input Focus Ring)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Updated input focus ring to emerald glow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Login/Login.css</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Category B (Light Mode Styling)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Merged (Select Focus Ring)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Updated select field focus ring to emerald glow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Exams/ExamsCenter.tsx</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Category A (Employee Role Page)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Merged (Full File)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Employee exam center view with assigned exams, answer submission, graded exam breakdown modal, and reviewer feedback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/CoursePlayer/CoursePlayer.tsx</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Category A (Employee Role Page)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Merged (Status Banner)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Employee course player completion status banner updated to brand emerald.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Admin/UserAdminStudio.tsx</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Category C (Admin/HR Studio)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Preserved Admin &amp; HR User Studio, role assignment, and department management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Creator/CreatorDashboard.tsx</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Category C (Manager/Admin Creator)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Preserved Creator Studio, course publishing/reverting, and approval queues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Reporting/ReportingDashboard.tsx</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Category C (Admin/HR Reporting)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Preserved 3-Level Department &amp; Employee Reporting analytics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Leaderboard/Leaderboard.tsx</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Category C (Leaderboard Page)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Preserved Leaderboard rankings and department filters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>frontend/src/components/Navbar/Navbar.tsx</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Category C (Shared Component)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Preserved Notification Bell badge, User Studio, Creator Studio, Reporting, and HR Manager navigation links.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Login/Login.tsx</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Category C (Auth &amp; Session)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Preserved HR Admin &amp; HR Manager session role mapping and department syncing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Backend &amp; API Files (app/*)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Category C (Backend Engine)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Preserved 91 active REST endpoints, RBAC permissions, audit logging, and notification triggers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>app/schemas/dashboard.py</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Backend Schema</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EmployeeDashboardResponse schema with exam_score_trend and category_progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>app/api/employee_dashboard.py</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Backend API Controller</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>GET /api/employee/dashboard endpoint calculating chronological score trends and status breakdowns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>frontend/src/components/Navbar/Navbar.tsx</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Navigation Links</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Hidden Leaderboard link and removed View Courses for Employee role.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>app/api/leaderboard.py</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Role Isolation</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Restricted Employee role from accessing GET /api/leaderboard (returns 403 Forbidden).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>app/api/employee_dashboard.py</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Department Scoping</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Restricted course categories and available courses strictly to employee own department.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Add Course selector to Exam Settings panel & fast template question parser
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Playwright E2E Verification" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Playwright E2E Verification" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -986,6 +986,33 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Item 15</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Step 15</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Exam Settings Course Selector &amp; Standalone Exam</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Added Department-filtered Course (Optional) selector in Exam Settings panel with None (Standalone Exam) option. Verified nullable course_id FK in DB and backend fallback across Attempt Exam, Reporting, Leaderboard, and Dashboard.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: resolve exam publish 500 error & integrate mandatory courses consistently into available lists
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Playwright E2E Verification" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Production Readiness Sprint" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47,8 +47,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F172A"/>
-        <bgColor rgb="000F172A"/>
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
       </patternFill>
     </fill>
     <fill>
@@ -463,30 +463,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>Phase</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Step #</t>
+          <t>Task / Feature</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Feature / Flow Description</t>
+          <t>Component Scope</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -496,520 +496,358 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Live Playwright Verification Details</t>
+          <t>Verification Details</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Item 1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Step 1</t>
+          <t>Phase 0</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Diagnostic Sweep &amp; Root Cause Analysis</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Restore Top Performing Department &amp; Remove Top Performing Learners</t>
+          <t>Full-stack Audit</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Re-added Top Performing Department hero card above BI grid and removed Top Performing Learners widget from Admin &amp; HR Dashboard.</t>
+          <t>Identified ADMIN role scoping bug, MCQ/MSQ schema gap, and missing AI department seed.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Item 2</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Step 2</t>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Core Flow Fix: Department creation -&gt; user section cascade</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Quiz Builder &amp; Notes Panel Right-Sizing</t>
+          <t>Backend / API</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Compacted .sidebar-tab-btn padding &amp; font size, trimmed .creator-notes-textarea min-height (120px), and right-sized question item padding.</t>
+          <t>Updated RequireRoles &amp; is_global_admin across dependencies, reporting, user_management.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Item 3</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Step 3</t>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Core Flow Fix: Courses page catalog rendering</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Course Cards Grid Clearance &amp; Overlap Fix</t>
+          <t>Frontend / Backend</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Applied grid-template-columns minmax(300px, 1fr), auto-rows minmax(320px, auto), gap 24px, and flex column layout to creator-course-card.</t>
+          <t>Mapped 'published' status to approved catalog items in ViewCourses.tsx &amp; course_service.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Item 4</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Step 4</t>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Core Flow Fix: Reporting page visibility for Admin</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>User Studio Delete Removal (Keep ONLY in Reporting)</t>
+          <t>Backend / API</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Removed delete buttons &amp; confirmation modals from UserStudio. Delete capability lives exclusively in Reporting -&gt; Employee Detail -&gt; Manage Employee.</t>
+          <t>Updated is_global_admin in reporting.py to recognize ADMIN role.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Item 5</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Step 5</t>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Core Flow Fix: MCQ &amp; MSQ question options &amp; auto-grading</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Exam Publish 500 Error Fix (MSQ Checkbox Questions)</t>
+          <t>Full-stack</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Sanitized non-UUID course_id &amp; department_id in ExamCreator.tsx and fixed is_published handling in app/api/exam.py.</t>
+          <t>Added options &amp; correct_answer JSON columns, radio/checkbox UI, and auto-scoring.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Item 6</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Step 6</t>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Database Hardening: FK indexes, constraints &amp; pooling</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Reporting Detail Profile 500 Error Fix (Users with Badges/Attempts)</t>
+          <t>Database / Alembic</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Fixed AttributeError on required_completions in app/api/reporting.py line 355. Profiles for users with attempts load cleanly with badge breakdown.</t>
+          <t>Applied migration f20000000001 with 11 B-tree FK indexes and pool_size=20.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Item 7</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Step 7</t>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Email OTP Integration: Hashed OTP, transactional email, 60s rate limit</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Notification Clear All &amp; Dismiss Persistence Fix</t>
+          <t>Auth / Services</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Added DELETE /api/notifications/clear-all &amp; DELETE /api/notifications/:id. Cleared notifications are deleted from DB so they never reappear on tab switch/reload.</t>
+          <t>PasswordResetOTP table, SMTP email service with fallback, 60s rate limit, and OTP UI.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Item 8</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Step 8</t>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory Courses: Auto-enrollment, visual badge, compliance widget</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Employee Dashboard Redesign (4 Personal Widgets)</t>
+          <t>Full-stack</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Replaced org-level stats with 4 personal widgets: My Avg Score &amp; Rank, Upcoming Exams, Learning Progress, and My Exam Score Trend.</t>
+          <t>is_mandatory column, Creator Studio toggle, auto-enrollment, badge, and compliance card.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Item 9</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Step 9</t>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>AI PDF Exam Generation: pypdf parsing, LLM/NLP prompt, staging review</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Standard Button Relabeling &amp; Review Mode</t>
+          <t>AI / Backend / UI</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Relabeled CTA buttons to Start Course / Continue Course / Review Course. Completed courses launch in Read-Only Review Mode with quiz retake locked.</t>
+          <t>AIExamService parsing, pending_ai_questions staging table, upload button &amp; review in ExamCreator.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Item 10</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Step 10</t>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Employee Leaderboard Tab: Department scoping &amp; self-rank highlighting</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Module Test Sequential Lock &amp; Gating</t>
+          <t>Frontend / API</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Advancing past module tests requires answering all questions. Next module remains locked until current test is submitted with a passing score.</t>
+          <t>Enabled Leaderboard link in Navbar for Employee, department scoping, (YOU) badge.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Item 11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Step 11</t>
+          <t>Phase 7</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Badge System Verification: Milestone triggers (courses &amp; exams)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Attempt Exam Navigation Tab</t>
+          <t>Backend / Services</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Added 'Attempt Exam' tab to top navbar for Employee role, linking to ExamsCenter (/exams) backed by real assigned exam API.</t>
+          <t>BadgeService milestone evaluation across course completions and graded exams.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Item 12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Step 12</t>
+          <t>Phase 8</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Seed AI Department Test Data: AI dept, 5 courses, 5 exams, 5 users</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Notification Auto-Mark-As-Read on Dropdown Open</t>
+          <t>Database / Seed</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Opening notification bell dropdown automatically fires PATCH /api/notifications/read-all, clearing unread badge count instantly.</t>
+          <t>Created seed_ai_department.py and seeded complete AI dataset with attempt history.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Item 13</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Step 13</t>
+          <t>Phase 9</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Console &amp; Network Cleanup</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>My Courses Multi-Course Loading Bug Fix</t>
+          <t>Full-stack Cleanup</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Root-caused bug in get_user_enrollments where status=='published' filter excluded status=='approved' courses. Fixed query so all mandatory and assigned courses load.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Item 14</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Step 14</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Manager Dashboard Rebuild (5 Department Widgets)</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Rebuilt Manager Dashboard with 5 widgets: Top Performer, Dept Avg Score, Top Course, Pass/Fail Donut, and Enrollment Trend Graphical Line Chart.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Item 15</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Step 15</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Backend Exam Scoping &amp; Visibility Fix</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>Fixed GET /api/exams in app/api/exam.py to correctly scope exams for Admin, HR, Manager, and Employee roles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Item 16</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Step 16</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Creator Studio Exams Catalog Tab &amp; HR Access</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Added Exams Catalog tab to CreatorDashboard.tsx listing all created exams with status badges and enabled HR_ADMIN role access.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Item 17</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Step 17</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Database Reset (Data-Only, Schema Preserved)</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Backed up DB to backup_before_reset_2026-07-26.sql, wiped all table data respecting FK constraints, preserved 1 root admin user (admin@lms.com), and verified empty-state handling live in Playwright Chromium.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Item 18</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Step 18</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Direct Role Creation &amp; Immediate Role Promotion Re-Scoping</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>Added User Role dropdown to Add User form, fixed Admin logout bug, added roles to UserResponse schema, enabled instant role sync in Navbar, and verified live end-to-end pass in Playwright Chromium.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Item 15</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Step 15</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Exam Settings Course Selector &amp; Standalone Exam</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Added Department-filtered Course (Optional) selector in Exam Settings panel with None (Standalone Exam) option. Verified nullable course_id FK in DB and backend fallback across Attempt Exam, Reporting, Leaderboard, and Dashboard.</t>
+          <t>Removed unused difficulty-distribution api call, fixed NameError in exams API for Employee/Manager, and cleaned up console logs.</t>
         </is>
       </c>
     </row>

</xml_diff>